<commit_message>
feat: automatiza fluxo completo de cancelamento
</commit_message>
<xml_diff>
--- a/planilhas/notas.xlsx
+++ b/planilhas/notas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BR0450988468\Desktop\bot-eorder\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B0FCE43-6030-4235-ABC5-42836705422C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E530195-F035-4A44-9F40-D41FC41BDD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="2250" windowWidth="14400" windowHeight="7280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1310" yWindow="1330" windowWidth="14400" windowHeight="7280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
     <t>29/06/2026 11:26</t>
   </si>
   <si>
-    <t>71005176690/001</t>
+    <t>71005173639/001</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat: adiciona loop para processar multiplas TdCs
</commit_message>
<xml_diff>
--- a/planilhas/notas.xlsx
+++ b/planilhas/notas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BR0450988468\Desktop\bot-eorder\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E530195-F035-4A44-9F40-D41FC41BDD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929CE324-6438-4282-8CBA-037AEE73314A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1310" yWindow="1330" windowWidth="14400" windowHeight="7280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
   <si>
     <t>CO</t>
   </si>
@@ -51,10 +51,22 @@
     <t/>
   </si>
   <si>
-    <t>29/06/2026 11:26</t>
-  </si>
-  <si>
-    <t>71005173639/001</t>
+    <t>19/06/2026 17:50</t>
+  </si>
+  <si>
+    <t>71005162958/001</t>
+  </si>
+  <si>
+    <t>19/06/2026 17:56</t>
+  </si>
+  <si>
+    <t>71005164531/001</t>
+  </si>
+  <si>
+    <t>19/06/2026 17:53</t>
+  </si>
+  <si>
+    <t>71005163653/001</t>
   </si>
 </sst>
 </file>
@@ -398,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
@@ -440,6 +452,40 @@
         <v>9</v>
       </c>
     </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>